<commit_message>
use built in serial pins, start on firmware using circuitpython
</commit_message>
<xml_diff>
--- a/layouts.xlsx
+++ b/layouts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cybdo\hackclub\CybdoClock\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28DD38F9-EDF3-421F-AEA7-5380002978B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED352683-B311-4415-971F-43A30C2D1402}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="3120" windowWidth="21600" windowHeight="11235" activeTab="1" xr2:uid="{45A766DE-614F-48DE-B5AD-AF16F24F84DB}"/>
+    <workbookView xWindow="9336" yWindow="5748" windowWidth="13704" windowHeight="7572" xr2:uid="{45A766DE-614F-48DE-B5AD-AF16F24F84DB}"/>
   </bookViews>
   <sheets>
     <sheet name="CLOCK" sheetId="1" r:id="rId1"/>
@@ -156,9 +156,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -495,623 +494,620 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C493D78-951E-49E6-99E7-866D65D92499}">
   <dimension ref="A1:N14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="16384" width="9.140625" style="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>14</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>23</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="1" t="s">
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s">
         <v>20</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>10</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="I1" s="1" t="s">
+      <c r="H1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I1" t="s">
         <v>20</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>21</v>
       </c>
-      <c r="K1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="M1" s="1" t="s">
+      <c r="K1" t="s">
+        <v>4</v>
+      </c>
+      <c r="L1" t="s">
+        <v>15</v>
+      </c>
+      <c r="M1" t="s">
         <v>13</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="1" t="s">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="F2" s="1" t="s">
+      <c r="D2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F2" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="J2" s="1" t="s">
+      <c r="G2" t="s">
+        <v>1</v>
+      </c>
+      <c r="H2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I2" t="s">
+        <v>4</v>
+      </c>
+      <c r="J2" t="s">
         <v>12</v>
       </c>
-      <c r="K2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="L2" s="1" t="s">
+      <c r="K2" t="s">
+        <v>3</v>
+      </c>
+      <c r="L2" t="s">
         <v>9</v>
       </c>
-      <c r="M2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="N2" s="1" t="s">
+      <c r="M2" t="s">
+        <v>1</v>
+      </c>
+      <c r="N2" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="1" t="s">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F3" s="1" t="s">
+      <c r="C3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E3" t="s">
+        <v>1</v>
+      </c>
+      <c r="F3" t="s">
         <v>14</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="G3" t="s">
         <v>22</v>
       </c>
-      <c r="H3" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="I3" s="1" t="s">
+      <c r="H3" t="s">
+        <v>1</v>
+      </c>
+      <c r="I3" t="s">
         <v>8</v>
       </c>
-      <c r="J3" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="K3" s="1" t="s">
+      <c r="J3" t="s">
+        <v>0</v>
+      </c>
+      <c r="K3" t="s">
         <v>9</v>
       </c>
-      <c r="L3" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="M3" s="1" t="s">
+      <c r="L3" t="s">
+        <v>1</v>
+      </c>
+      <c r="M3" t="s">
         <v>14</v>
       </c>
-      <c r="N3" s="1" t="s">
+      <c r="N3" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="A4" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" s="1" t="s">
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="F4" s="1" t="s">
+      <c r="E4" t="s">
+        <v>0</v>
+      </c>
+      <c r="F4" t="s">
         <v>12</v>
       </c>
-      <c r="G4" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="H4" s="1" t="s">
+      <c r="G4" t="s">
+        <v>1</v>
+      </c>
+      <c r="H4" t="s">
         <v>14</v>
       </c>
-      <c r="I4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="K4" s="1" t="s">
+      <c r="I4" t="s">
+        <v>3</v>
+      </c>
+      <c r="J4" t="s">
+        <v>1</v>
+      </c>
+      <c r="K4" t="s">
         <v>6</v>
       </c>
-      <c r="L4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="M4" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="N4" s="1" t="s">
+      <c r="L4" t="s">
+        <v>3</v>
+      </c>
+      <c r="M4" t="s">
+        <v>4</v>
+      </c>
+      <c r="N4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="A5" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D5" s="1" t="s">
+      <c r="C5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G5" s="1" t="s">
+      <c r="E5" t="s">
+        <v>1</v>
+      </c>
+      <c r="F5" t="s">
+        <v>5</v>
+      </c>
+      <c r="G5" t="s">
         <v>9</v>
       </c>
-      <c r="H5" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="J5" s="1" t="s">
+      <c r="H5" t="s">
+        <v>2</v>
+      </c>
+      <c r="I5" t="s">
+        <v>0</v>
+      </c>
+      <c r="J5" t="s">
         <v>17</v>
       </c>
-      <c r="K5" s="1" t="s">
+      <c r="K5" t="s">
         <v>12</v>
       </c>
-      <c r="L5" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="M5" s="1" t="s">
+      <c r="L5" t="s">
+        <v>3</v>
+      </c>
+      <c r="M5" t="s">
         <v>13</v>
       </c>
-      <c r="N5" s="1" t="s">
+      <c r="N5" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="A6" t="s">
         <v>20</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D6" s="1" t="s">
+      <c r="B6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" t="s">
         <v>11</v>
       </c>
-      <c r="E6" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="J6" s="1" t="s">
+      <c r="E6" t="s">
+        <v>5</v>
+      </c>
+      <c r="F6" t="s">
+        <v>4</v>
+      </c>
+      <c r="G6" t="s">
+        <v>0</v>
+      </c>
+      <c r="H6" t="s">
+        <v>4</v>
+      </c>
+      <c r="I6" t="s">
+        <v>5</v>
+      </c>
+      <c r="J6" t="s">
         <v>10</v>
       </c>
-      <c r="K6" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="L6" s="1" t="s">
+      <c r="K6" t="s">
+        <v>5</v>
+      </c>
+      <c r="L6" t="s">
         <v>11</v>
       </c>
-      <c r="M6" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="N6" s="1" t="s">
+      <c r="M6" t="s">
+        <v>5</v>
+      </c>
+      <c r="N6" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B7" s="1" t="s">
+      <c r="A7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B7" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" t="s">
         <v>9</v>
       </c>
-      <c r="D7" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="G7" s="1" t="s">
+      <c r="D7" t="s">
+        <v>5</v>
+      </c>
+      <c r="E7" t="s">
+        <v>5</v>
+      </c>
+      <c r="F7" t="s">
+        <v>0</v>
+      </c>
+      <c r="G7" t="s">
         <v>7</v>
       </c>
-      <c r="H7" s="1" t="s">
+      <c r="H7" t="s">
         <v>8</v>
       </c>
-      <c r="I7" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="J7" s="1" t="s">
+      <c r="I7" t="s">
+        <v>1</v>
+      </c>
+      <c r="J7" t="s">
         <v>10</v>
       </c>
-      <c r="K7" s="1" t="s">
+      <c r="K7" t="s">
         <v>12</v>
       </c>
-      <c r="L7" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="M7" s="1" t="s">
+      <c r="L7" t="s">
+        <v>0</v>
+      </c>
+      <c r="M7" t="s">
         <v>11</v>
       </c>
-      <c r="N7" s="1" t="s">
+      <c r="N7" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F8" s="1" t="s">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>1</v>
+      </c>
+      <c r="C8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" t="s">
+        <v>5</v>
+      </c>
+      <c r="E8" t="s">
+        <v>4</v>
+      </c>
+      <c r="F8" t="s">
         <v>20</v>
       </c>
-      <c r="G8" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="I8" s="1" t="s">
+      <c r="G8" t="s">
+        <v>1</v>
+      </c>
+      <c r="H8" t="s">
+        <v>3</v>
+      </c>
+      <c r="I8" t="s">
         <v>21</v>
       </c>
-      <c r="J8" s="1" t="s">
+      <c r="J8" t="s">
         <v>18</v>
       </c>
-      <c r="K8" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="L8" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="M8" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="N8" s="1" t="s">
+      <c r="K8" t="s">
+        <v>15</v>
+      </c>
+      <c r="L8" t="s">
+        <v>2</v>
+      </c>
+      <c r="M8" t="s">
+        <v>1</v>
+      </c>
+      <c r="N8" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B9" s="1" t="s">
+      <c r="A9" t="s">
+        <v>1</v>
+      </c>
+      <c r="B9" t="s">
         <v>8</v>
       </c>
-      <c r="C9" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D9" s="1" t="s">
+      <c r="C9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" t="s">
         <v>20</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="E9" t="s">
         <v>21</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="F9" t="s">
         <v>18</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="G9" t="s">
         <v>20</v>
       </c>
-      <c r="H9" s="1" t="s">
+      <c r="H9" t="s">
         <v>10</v>
       </c>
-      <c r="I9" s="1" t="s">
+      <c r="I9" t="s">
         <v>13</v>
       </c>
-      <c r="J9" s="1" t="s">
+      <c r="J9" t="s">
         <v>22</v>
       </c>
-      <c r="K9" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="L9" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="M9" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="N9" s="1" t="s">
+      <c r="K9" t="s">
+        <v>15</v>
+      </c>
+      <c r="L9" t="s">
+        <v>3</v>
+      </c>
+      <c r="M9" t="s">
+        <v>4</v>
+      </c>
+      <c r="N9" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="H10" s="1" t="s">
+      <c r="A10" t="s">
+        <v>1</v>
+      </c>
+      <c r="B10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C10" t="s">
+        <v>4</v>
+      </c>
+      <c r="D10" t="s">
+        <v>0</v>
+      </c>
+      <c r="E10" t="s">
+        <v>4</v>
+      </c>
+      <c r="F10" t="s">
+        <v>5</v>
+      </c>
+      <c r="G10" t="s">
+        <v>0</v>
+      </c>
+      <c r="H10" t="s">
         <v>7</v>
       </c>
-      <c r="I10" s="1" t="s">
+      <c r="I10" t="s">
         <v>8</v>
       </c>
-      <c r="J10" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="K10" s="1" t="s">
+      <c r="J10" t="s">
+        <v>1</v>
+      </c>
+      <c r="K10" t="s">
         <v>6</v>
       </c>
-      <c r="L10" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="M10" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="N10" s="1" t="s">
+      <c r="L10" t="s">
+        <v>3</v>
+      </c>
+      <c r="M10" t="s">
+        <v>4</v>
+      </c>
+      <c r="N10" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" s="1" t="s">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
         <v>12</v>
       </c>
-      <c r="C11" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D11" s="1" t="s">
+      <c r="C11" t="s">
+        <v>3</v>
+      </c>
+      <c r="D11" t="s">
         <v>13</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="E11" t="s">
         <v>9</v>
       </c>
-      <c r="F11" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H11" s="1" t="s">
+      <c r="F11" t="s">
+        <v>2</v>
+      </c>
+      <c r="G11" t="s">
+        <v>5</v>
+      </c>
+      <c r="H11" t="s">
         <v>11</v>
       </c>
-      <c r="I11" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="J11" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="K11" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="L11" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="M11" s="1" t="s">
+      <c r="I11" t="s">
+        <v>5</v>
+      </c>
+      <c r="J11" t="s">
+        <v>4</v>
+      </c>
+      <c r="K11" t="s">
+        <v>2</v>
+      </c>
+      <c r="L11" t="s">
+        <v>0</v>
+      </c>
+      <c r="M11" t="s">
         <v>17</v>
       </c>
-      <c r="N11" s="1" t="s">
+      <c r="N11" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
+      <c r="A12" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C12" s="1" t="s">
+      <c r="B12" t="s">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
         <v>11</v>
       </c>
-      <c r="D12" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E12" s="1" t="s">
+      <c r="D12" t="s">
+        <v>5</v>
+      </c>
+      <c r="E12" t="s">
         <v>10</v>
       </c>
-      <c r="F12" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G12" s="1" t="s">
+      <c r="F12" t="s">
+        <v>5</v>
+      </c>
+      <c r="G12" t="s">
         <v>11</v>
       </c>
-      <c r="H12" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="I12" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="J12" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="K12" s="1" t="s">
+      <c r="H12" t="s">
+        <v>5</v>
+      </c>
+      <c r="I12" t="s">
+        <v>4</v>
+      </c>
+      <c r="J12" t="s">
+        <v>1</v>
+      </c>
+      <c r="K12" t="s">
         <v>8</v>
       </c>
-      <c r="L12" s="1" t="s">
+      <c r="L12" t="s">
         <v>9</v>
       </c>
-      <c r="M12" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="N12" s="1" t="s">
+      <c r="M12" t="s">
+        <v>5</v>
+      </c>
+      <c r="N12" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B13" s="1" t="s">
+      <c r="A13" t="s">
+        <v>1</v>
+      </c>
+      <c r="B13" t="s">
         <v>6</v>
       </c>
-      <c r="C13" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D13" s="1" t="s">
+      <c r="C13" t="s">
+        <v>5</v>
+      </c>
+      <c r="D13" t="s">
         <v>10</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="E13" t="s">
         <v>11</v>
       </c>
-      <c r="F13" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H13" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="I13" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="J13" s="1" t="s">
+      <c r="F13" t="s">
+        <v>5</v>
+      </c>
+      <c r="G13" t="s">
+        <v>5</v>
+      </c>
+      <c r="H13" t="s">
+        <v>3</v>
+      </c>
+      <c r="I13" t="s">
+        <v>4</v>
+      </c>
+      <c r="J13" t="s">
         <v>20</v>
       </c>
-      <c r="K13" s="1" t="s">
+      <c r="K13" t="s">
         <v>10</v>
       </c>
-      <c r="L13" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="M13" s="1" t="s">
+      <c r="L13" t="s">
+        <v>3</v>
+      </c>
+      <c r="M13" t="s">
         <v>20</v>
       </c>
-      <c r="N13" s="1" t="s">
+      <c r="N13" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
+      <c r="A14" t="s">
         <v>18</v>
       </c>
-      <c r="B14" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C14" s="1" t="s">
+      <c r="B14" t="s">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
         <v>12</v>
       </c>
-      <c r="D14" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E14" s="1" t="s">
+      <c r="D14" t="s">
+        <v>15</v>
+      </c>
+      <c r="E14" t="s">
         <v>10</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="F14" t="s">
         <v>10</v>
       </c>
-      <c r="G14" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="H14" s="1" t="s">
+      <c r="G14" t="s">
+        <v>3</v>
+      </c>
+      <c r="H14" t="s">
         <v>13</v>
       </c>
-      <c r="I14" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="J14" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="K14" s="1" t="s">
+      <c r="I14" t="s">
+        <v>1</v>
+      </c>
+      <c r="J14" t="s">
+        <v>15</v>
+      </c>
+      <c r="K14" t="s">
         <v>18</v>
       </c>
-      <c r="L14" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="M14" s="1" t="s">
+      <c r="L14" t="s">
+        <v>4</v>
+      </c>
+      <c r="M14" t="s">
         <v>23</v>
       </c>
-      <c r="N14" s="1" t="s">
+      <c r="N14" t="s">
         <v>21</v>
       </c>
     </row>

</xml_diff>

<commit_message>
firmware done, centered leds positioning
</commit_message>
<xml_diff>
--- a/layouts.xlsx
+++ b/layouts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cybdo\hackclub\CybdoClock\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED352683-B311-4415-971F-43A30C2D1402}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46455349-78A1-48A0-897A-829F49CAED3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9336" yWindow="5748" windowWidth="13704" windowHeight="7572" xr2:uid="{45A766DE-614F-48DE-B5AD-AF16F24F84DB}"/>
+    <workbookView xWindow="4308" yWindow="2736" windowWidth="14652" windowHeight="9048" xr2:uid="{45A766DE-614F-48DE-B5AD-AF16F24F84DB}"/>
   </bookViews>
   <sheets>
     <sheet name="CLOCK" sheetId="1" r:id="rId1"/>
@@ -136,12 +136,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -156,8 +162,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -788,13 +795,13 @@
         <v>1</v>
       </c>
       <c r="J7" t="s">
+        <v>6</v>
+      </c>
+      <c r="K7" t="s">
+        <v>5</v>
+      </c>
+      <c r="L7" t="s">
         <v>10</v>
-      </c>
-      <c r="K7" t="s">
-        <v>12</v>
-      </c>
-      <c r="L7" t="s">
-        <v>0</v>
       </c>
       <c r="M7" t="s">
         <v>11</v>
@@ -804,91 +811,91 @@
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" t="s">
-        <v>1</v>
-      </c>
-      <c r="C8" t="s">
-        <v>5</v>
-      </c>
-      <c r="D8" t="s">
-        <v>5</v>
-      </c>
-      <c r="E8" t="s">
-        <v>4</v>
-      </c>
-      <c r="F8" t="s">
+      <c r="A8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="G8" t="s">
-        <v>1</v>
-      </c>
-      <c r="H8" t="s">
-        <v>3</v>
-      </c>
-      <c r="I8" t="s">
+      <c r="F8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="L8" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="M8" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="J8" t="s">
+      <c r="N8" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F9" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="K8" t="s">
-        <v>15</v>
-      </c>
-      <c r="L8" t="s">
-        <v>2</v>
-      </c>
-      <c r="M8" t="s">
-        <v>1</v>
-      </c>
-      <c r="N8" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>1</v>
-      </c>
-      <c r="B9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C9" t="s">
-        <v>15</v>
-      </c>
-      <c r="D9" t="s">
+      <c r="G9" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="E9" t="s">
-        <v>21</v>
-      </c>
-      <c r="F9" t="s">
+      <c r="H9" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="K9" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="G9" t="s">
-        <v>20</v>
-      </c>
-      <c r="H9" t="s">
-        <v>10</v>
-      </c>
-      <c r="I9" t="s">
-        <v>13</v>
-      </c>
-      <c r="J9" t="s">
-        <v>22</v>
-      </c>
-      <c r="K9" t="s">
-        <v>15</v>
-      </c>
-      <c r="L9" t="s">
-        <v>3</v>
-      </c>
-      <c r="M9" t="s">
-        <v>4</v>
-      </c>
-      <c r="N9" t="s">
-        <v>21</v>
+      <c r="L9" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="M9" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="N9" s="1" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">

</xml_diff>